<commit_message>
swapped out utility/region for avoided_cost_subset in all demo data input files
</commit_message>
<xml_diff>
--- a/profiles/demo/data/custom_gas_load_shapes.xlsx
+++ b/profiles/demo/data/custom_gas_load_shapes.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>month</t>
   </si>
@@ -38,6 +38,9 @@
   </si>
   <si>
     <t>hpwh_electrification_therms_impact_norm</t>
+  </si>
+  <si>
+    <t>hpwh_electrification_therms_savings</t>
   </si>
 </sst>
 </file>
@@ -346,7 +349,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="2">

</xml_diff>

<commit_message>
region,utility -> avoided cost subset
* swapped out utility/region for avoided_cost_subset in all demo data input files

* replace the notion of region/utility by avoided_cost_subset in the SQL code

* replace the notion of region/utility by avoided_cost_subset in the SQL code

---------

Co-authored-by: loic <loic.fontaine@recurve.com>
</commit_message>
<xml_diff>
--- a/profiles/demo/data/custom_gas_load_shapes.xlsx
+++ b/profiles/demo/data/custom_gas_load_shapes.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>month</t>
   </si>
@@ -38,6 +38,9 @@
   </si>
   <si>
     <t>hpwh_electrification_therms_impact_norm</t>
+  </si>
+  <si>
+    <t>hpwh_electrification_therms_savings</t>
   </si>
 </sst>
 </file>
@@ -346,7 +349,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="2">

</xml_diff>